<commit_message>
Fix Tableau cash flow export
</commit_message>
<xml_diff>
--- a/dashboard/PANW_3Statement_Model.xlsx
+++ b/dashboard/PANW_3Statement_Model.xlsx
@@ -16,7 +16,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt_Schedule" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue_Disaggregation" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +28,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;d&quot;"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,23 +95,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FF0000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <i val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
+      <color rgb="00375623"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -166,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,21 +193,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -607,7 +575,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-24</t>
+          <t>Generated: 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -629,136 +597,6 @@
 • BalanceCheck tolerance: $1M. Cash is the balancing item derived from the CF statement — NOT set independently.
 • Full SaaS-grade modeling (deferred-revenue dynamics, OCI components, debt-schedule embedded options) is v2 work.
 • Source: SEC EDGAR XBRL facts. Provenance on the Sources sheet — every value traces to an accession number.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B1:B21"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="85" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="29" t="inlineStr">
-        <is>
-          <t>PANW Revenue Disaggregation — ASC 280 Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="30" t="inlineStr">
-        <is>
-          <t>SEGMENT REPORTING (ASC 280)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="31" t="inlineStr">
-        <is>
-          <t>PANW reports as ONE operating and reportable segment under ASC 280. There are no separately reportable segments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>REVENUE DISAGGREGATION (ASC 606)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="31" t="inlineStr">
-        <is>
-          <t>Revenue is disaggregated into TWO categories in the 10-K:</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. Product  — next-gen firewall appliances and other hardware</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. Subscription and Support (S&amp;S)  — cloud subscriptions, software updates, premium support, maintenance</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>PRODUCT FAMILIES (commercial brands, NOT segments)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="B12" s="31" t="inlineStr">
-        <is>
-          <t>Strata, Prisma, and Cortex are product families — commercial brands that span both revenue categories:</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="34" customHeight="1">
-      <c r="B13" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Strata  — generates both Product revenue (from firewall appliances) AND S&amp;S revenue (from subscriptions running on those appliances)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="B14" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Prisma  — cloud-delivered SASE/CNAPP; almost entirely S&amp;S</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="B15" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Cortex  — XDR/XSIAM; almost entirely S&amp;S</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="B16" s="32" t="inlineStr">
-        <is>
-          <t>Calling Strata/Prisma/Cortex 'segments' is incorrect under ASC 280.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="B18" s="30" t="inlineStr">
-        <is>
-          <t>CURRENT MODEL SCOPE</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="67" customHeight="1">
-      <c r="B19" s="31" t="inlineStr">
-        <is>
-          <t>This model forecasts CONSOLIDATED REVENUE only. Disaggregating into Product vs. Subscription &amp; Support is a v2 enhancement; disaggregating further by product family would require parsing narrative text from earnings releases (XBRL does not tag it at that granularity).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="45" customHeight="1">
-      <c r="B21" s="33" t="inlineStr">
-        <is>
-          <t>Forecasting Product and Subscription &amp; Support separately is a v2 enhancement. NGS ARR — PANW's headline non-GAAP metric — is not exposed as structured XBRL and is out of scope here.</t>
         </is>
       </c>
     </row>
@@ -811,13 +649,13 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>-0.2</v>
+        <v>0.04</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>-0.3</v>
+        <v>0.06</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>-0.08000000000000002</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="3">
@@ -859,13 +697,13 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>0.001</v>
+        <v>0.07870791628753412</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>0.001</v>
+        <v>0.07870791628753412</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>0.001</v>
+        <v>0.07870791628753412</v>
       </c>
     </row>
     <row r="6">
@@ -898,22 +736,6 @@
       </c>
       <c r="D7" s="7" t="n">
         <v>45</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>DIO (days)</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -998,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1042,7 +864,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>-0.2</v>
+        <v>0.04</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -1087,7 +909,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>0.001</v>
+        <v>0.07870791628753412</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -1128,73 +950,58 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>DIO (days)</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="n">
-        <v>0</v>
+          <t>Effective Tax Rate</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>0.15</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Days Inventory Outstanding — drives Inventory = (DIO/90) × COGS</t>
+          <t>Applied to positive PreTax Income only</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Effective Tax Rate</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="n">
-        <v>0.15</v>
+          <t>Debt Amortization Qtrly</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Applied to positive PreTax Income only</t>
+          <t>Mandatory quarterly principal repayment</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Debt Amortization Qtrly</t>
+          <t>SBC Quarterly ($)</t>
         </is>
       </c>
       <c r="B11" s="14" t="n">
-        <v>0</v>
+        <v>615000000</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Mandatory quarterly principal repayment</t>
+          <t>Non-cash OCF add-back; held flat at latest historical value</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>SBC Quarterly ($)</t>
+          <t>Buybacks Quarterly ($)</t>
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Non-cash OCF add-back; held flat at latest historical value</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Buybacks Quarterly ($)</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Financing-line cash outflow; held flat at latest historical value</t>
         </is>
@@ -1334,26 +1141,24 @@
       <c r="B2" s="16" t="n">
         <v>6685200000</v>
       </c>
-      <c r="C2" s="16" t="n">
-        <v>5838000000</v>
-      </c>
+      <c r="C2" s="17" t="n"/>
       <c r="D2" s="16" t="n">
+        <v>2474000000</v>
+      </c>
+      <c r="E2" s="17" t="n"/>
+      <c r="F2" s="17" t="n"/>
+      <c r="G2" s="16" t="n">
         <v>2139000000</v>
       </c>
-      <c r="E2" s="16" t="n">
-        <v>2474000000</v>
-      </c>
-      <c r="F2" s="17" t="n"/>
-      <c r="G2" s="17" t="n"/>
-      <c r="H2" s="17" t="n"/>
-      <c r="I2" s="16" t="n">
+      <c r="H2" s="16" t="n">
         <v>5068000000</v>
       </c>
-      <c r="J2" s="17" t="n"/>
+      <c r="I2" s="17" t="n"/>
+      <c r="J2" s="16" t="n">
+        <v>4396000000</v>
+      </c>
       <c r="K2" s="17" t="n"/>
-      <c r="L2" s="16" t="n">
-        <v>4396000000</v>
-      </c>
+      <c r="L2" s="17" t="n"/>
       <c r="M2" s="17" t="n"/>
       <c r="N2" s="18" t="n">
         <v>0</v>
@@ -1377,26 +1182,24 @@
       <c r="B3" s="16" t="n">
         <v>1772600000</v>
       </c>
-      <c r="C3" s="16" t="n">
-        <v>1485500000</v>
-      </c>
+      <c r="C3" s="17" t="n"/>
       <c r="D3" s="16" t="n">
+        <v>638000000</v>
+      </c>
+      <c r="E3" s="17" t="n"/>
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="16" t="n">
         <v>554000000</v>
       </c>
-      <c r="E3" s="16" t="n">
-        <v>638000000</v>
-      </c>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="17" t="n"/>
-      <c r="H3" s="17" t="n"/>
-      <c r="I3" s="16" t="n">
+      <c r="H3" s="16" t="n">
         <v>1323000000</v>
       </c>
-      <c r="J3" s="17" t="n"/>
+      <c r="I3" s="17" t="n"/>
+      <c r="J3" s="16" t="n">
+        <v>1153000000</v>
+      </c>
       <c r="K3" s="17" t="n"/>
-      <c r="L3" s="16" t="n">
-        <v>1153000000</v>
-      </c>
+      <c r="L3" s="17" t="n"/>
       <c r="M3" s="17" t="n"/>
       <c r="N3" s="18" t="n">
         <v>0</v>
@@ -1420,26 +1223,24 @@
       <c r="B4" s="16" t="n">
         <v>4912600000</v>
       </c>
-      <c r="C4" s="16" t="n">
-        <v>4352500000</v>
-      </c>
+      <c r="C4" s="17" t="n"/>
       <c r="D4" s="16" t="n">
+        <v>1836000000</v>
+      </c>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="16" t="n">
         <v>1585000000</v>
       </c>
-      <c r="E4" s="16" t="n">
-        <v>1836000000</v>
-      </c>
-      <c r="F4" s="17" t="n"/>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="17" t="n"/>
-      <c r="I4" s="16" t="n">
+      <c r="H4" s="16" t="n">
         <v>3745000000</v>
       </c>
-      <c r="J4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="16" t="n">
+        <v>3243000000</v>
+      </c>
       <c r="K4" s="17" t="n"/>
-      <c r="L4" s="16" t="n">
-        <v>3243000000</v>
-      </c>
+      <c r="L4" s="17" t="n"/>
       <c r="M4" s="17" t="n"/>
       <c r="N4" s="18" t="n">
         <v>0</v>
@@ -1463,26 +1264,24 @@
       <c r="B5" s="16" t="n">
         <v>4166900000</v>
       </c>
-      <c r="C5" s="16" t="n">
-        <v>3907000000</v>
-      </c>
+      <c r="C5" s="17" t="n"/>
       <c r="D5" s="16" t="n">
+        <v>1527000000</v>
+      </c>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="16" t="n">
         <v>1299000000</v>
       </c>
-      <c r="E5" s="16" t="n">
-        <v>1527000000</v>
-      </c>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="16" t="n">
+      <c r="H5" s="16" t="n">
         <v>3039000000</v>
       </c>
-      <c r="J5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="16" t="n">
+        <v>2716000000</v>
+      </c>
       <c r="K5" s="17" t="n"/>
-      <c r="L5" s="16" t="n">
-        <v>2716000000</v>
-      </c>
+      <c r="L5" s="17" t="n"/>
       <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
         <v>0</v>
@@ -1506,26 +1305,24 @@
       <c r="B6" s="16" t="n">
         <v>745700000</v>
       </c>
-      <c r="C6" s="16" t="n">
-        <v>445500000</v>
-      </c>
+      <c r="C6" s="17" t="n"/>
       <c r="D6" s="16" t="n">
+        <v>309000000</v>
+      </c>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="16" t="n">
         <v>286000000</v>
       </c>
-      <c r="E6" s="16" t="n">
-        <v>309000000</v>
-      </c>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="16" t="n">
+      <c r="H6" s="16" t="n">
         <v>706000000</v>
       </c>
-      <c r="J6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="16" t="n">
+        <v>527000000</v>
+      </c>
       <c r="K6" s="17" t="n"/>
-      <c r="L6" s="16" t="n">
-        <v>527000000</v>
-      </c>
+      <c r="L6" s="17" t="n"/>
       <c r="M6" s="17" t="n"/>
       <c r="N6" s="18" t="n">
         <v>0</v>
@@ -1549,26 +1346,24 @@
       <c r="B7" s="16" t="n">
         <v>880100000</v>
       </c>
-      <c r="C7" s="16" t="n">
-        <v>2219900000</v>
-      </c>
+      <c r="C7" s="17" t="n"/>
       <c r="D7" s="16" t="n">
+        <v>334000000</v>
+      </c>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="16" t="n">
         <v>351000000</v>
       </c>
-      <c r="E7" s="16" t="n">
-        <v>334000000</v>
-      </c>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="16" t="n">
+      <c r="H7" s="16" t="n">
         <v>766000000</v>
       </c>
-      <c r="J7" s="17" t="n"/>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="16" t="n">
+        <v>618000000</v>
+      </c>
       <c r="K7" s="17" t="n"/>
-      <c r="L7" s="16" t="n">
-        <v>618000000</v>
-      </c>
+      <c r="L7" s="17" t="n"/>
       <c r="M7" s="17" t="n"/>
       <c r="N7" s="18" t="n">
         <v>0</v>
@@ -1592,19 +1387,16 @@
       <c r="B9" s="19" t="n">
         <v>0.7348471249925208</v>
       </c>
-      <c r="C9" s="19" t="n">
-        <v>0.7455464200068517</v>
-      </c>
       <c r="D9" s="19" t="n">
+        <v>0.7421180274858529</v>
+      </c>
+      <c r="G9" s="19" t="n">
         <v>0.7410004675081814</v>
       </c>
-      <c r="E9" s="19" t="n">
-        <v>0.7421180274858529</v>
-      </c>
-      <c r="I9" s="19" t="n">
+      <c r="H9" s="19" t="n">
         <v>0.738950276243094</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="J9" s="19" t="n">
         <v>0.7377161055505005</v>
       </c>
       <c r="N9" s="20" t="n">
@@ -1631,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1754,10 +1546,10 @@
         <v>1346300000</v>
       </c>
       <c r="F3" s="16" t="n">
+        <v>1992900000</v>
+      </c>
+      <c r="G3" s="16" t="n">
         <v>2118500000</v>
-      </c>
-      <c r="G3" s="16" t="n">
-        <v>1992900000</v>
       </c>
       <c r="H3" s="16" t="n">
         <v>1373700000</v>
@@ -1766,10 +1558,10 @@
         <v>2383400000</v>
       </c>
       <c r="J3" s="16" t="n">
+        <v>2269000000</v>
+      </c>
+      <c r="K3" s="16" t="n">
         <v>3066000000</v>
-      </c>
-      <c r="K3" s="16" t="n">
-        <v>2269000000</v>
       </c>
       <c r="L3" s="16" t="n">
         <v>2269000000</v>
@@ -1805,10 +1597,10 @@
         <v>1278100000</v>
       </c>
       <c r="F4" s="16" t="n">
+        <v>1443600000</v>
+      </c>
+      <c r="G4" s="16" t="n">
         <v>2142500000</v>
-      </c>
-      <c r="G4" s="16" t="n">
-        <v>1443600000</v>
       </c>
       <c r="H4" s="16" t="n">
         <v>1715400000</v>
@@ -1817,10 +1609,10 @@
         <v>1950000000</v>
       </c>
       <c r="J4" s="16" t="n">
+        <v>2965000000</v>
+      </c>
+      <c r="K4" s="16" t="n">
         <v>1343000000</v>
-      </c>
-      <c r="K4" s="16" t="n">
-        <v>2965000000</v>
       </c>
       <c r="L4" s="16" t="n">
         <v>2965000000</v>
@@ -1844,319 +1636,288 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Inventory</t>
+          <t>TOTAL ASSETS</t>
         </is>
       </c>
       <c r="B5" s="17" t="n"/>
       <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
+      <c r="D5" s="16" t="n">
+        <v>12543800000</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>13163400000</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>14170500000</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>12253600000</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>17930800000</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>22002800000</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>23576000000</v>
+      </c>
+      <c r="K5" s="16" t="n">
+        <v>23536000000</v>
+      </c>
+      <c r="L5" s="16" t="n">
+        <v>23576000000</v>
+      </c>
+      <c r="M5" s="16" t="n">
+        <v>24979000000</v>
+      </c>
       <c r="N5" s="18" t="n">
-        <v>0</v>
+        <v>25332000000</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>0</v>
+        <v>25947000000</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>0</v>
+        <v>26562000000</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL ASSETS</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="16" t="n">
-        <v>12543800000</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>13163400000</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <v>12253600000</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>14170500000</v>
-      </c>
-      <c r="H6" s="16" t="n">
-        <v>17930800000</v>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>22002800000</v>
-      </c>
-      <c r="J6" s="16" t="n">
-        <v>23536000000</v>
-      </c>
-      <c r="K6" s="16" t="n">
-        <v>23576000000</v>
-      </c>
-      <c r="L6" s="16" t="n">
-        <v>23576000000</v>
-      </c>
-      <c r="M6" s="16" t="n">
-        <v>24979000000</v>
-      </c>
-      <c r="N6" s="18" t="n">
-        <v>25332000000</v>
-      </c>
-      <c r="O6" s="18" t="n">
-        <v>25947000000</v>
-      </c>
-      <c r="P6" s="18" t="n">
-        <v>26562000000</v>
-      </c>
-      <c r="Q6" s="18" t="n">
         <v>27177000000</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>LIABILITIES</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>LIABILITIES</t>
-        </is>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Accounts Payable</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="16" t="n">
+        <v>125900000</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>128300000</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>91600000</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>128000000</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>108900000</v>
+      </c>
+      <c r="I8" s="16" t="n">
+        <v>234800000</v>
+      </c>
+      <c r="J8" s="16" t="n">
+        <v>232000000</v>
+      </c>
+      <c r="K8" s="16" t="n">
+        <v>223000000</v>
+      </c>
+      <c r="L8" s="16" t="n">
+        <v>232000000</v>
+      </c>
+      <c r="M8" s="16" t="n">
+        <v>262000000</v>
+      </c>
+      <c r="N8" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Deferred Revenue</t>
         </is>
       </c>
       <c r="B9" s="17" t="n"/>
       <c r="C9" s="17" t="n"/>
       <c r="D9" s="16" t="n">
-        <v>125900000</v>
+        <v>3741300000</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>128300000</v>
+        <v>3942500000</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>128000000</v>
+        <v>4146700000</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>91600000</v>
+        <v>3641200000</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>108900000</v>
+        <v>5014900000</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>234800000</v>
+        <v>5756800000</v>
       </c>
       <c r="J9" s="16" t="n">
-        <v>223000000</v>
+        <v>6302000000</v>
       </c>
       <c r="K9" s="16" t="n">
-        <v>232000000</v>
+        <v>6132000000</v>
       </c>
       <c r="L9" s="16" t="n">
-        <v>232000000</v>
+        <v>6302000000</v>
       </c>
       <c r="M9" s="16" t="n">
-        <v>262000000</v>
+        <v>6248000000</v>
       </c>
       <c r="N9" s="18" t="n">
-        <v>0</v>
+        <v>6248000000</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>0</v>
+        <v>6248000000</v>
       </c>
       <c r="P9" s="18" t="n">
-        <v>0</v>
+        <v>6248000000</v>
       </c>
       <c r="Q9" s="18" t="n">
-        <v>0</v>
+        <v>6248000000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Deferred Revenue</t>
+          <t>TOTAL LIABILITIES</t>
         </is>
       </c>
       <c r="B10" s="17" t="n"/>
       <c r="C10" s="17" t="n"/>
       <c r="D10" s="16" t="n">
-        <v>3741300000</v>
+        <v>12035800000</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>3942500000</v>
+        <v>12434400000</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>3641200000</v>
+        <v>12938100000</v>
       </c>
       <c r="G10" s="16" t="n">
-        <v>4146700000</v>
+        <v>12043600000</v>
       </c>
       <c r="H10" s="16" t="n">
-        <v>5014900000</v>
+        <v>13463000000</v>
       </c>
       <c r="I10" s="16" t="n">
-        <v>5756800000</v>
+        <v>14772300000</v>
       </c>
       <c r="J10" s="16" t="n">
-        <v>6132000000</v>
+        <v>15752000000</v>
       </c>
       <c r="K10" s="16" t="n">
-        <v>6302000000</v>
+        <v>14871000000</v>
       </c>
       <c r="L10" s="16" t="n">
-        <v>6302000000</v>
+        <v>15752000000</v>
       </c>
       <c r="M10" s="16" t="n">
-        <v>6248000000</v>
+        <v>15586000000</v>
       </c>
       <c r="N10" s="18" t="n">
-        <v>6248000000</v>
+        <v>15324000000</v>
       </c>
       <c r="O10" s="18" t="n">
-        <v>6248000000</v>
+        <v>15324000000</v>
       </c>
       <c r="P10" s="18" t="n">
-        <v>6248000000</v>
+        <v>15324000000</v>
       </c>
       <c r="Q10" s="18" t="n">
-        <v>6248000000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL LIABILITIES</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="16" t="n">
-        <v>12035800000</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <v>12434400000</v>
-      </c>
-      <c r="F11" s="16" t="n">
-        <v>12043600000</v>
-      </c>
-      <c r="G11" s="16" t="n">
-        <v>12938100000</v>
-      </c>
-      <c r="H11" s="16" t="n">
-        <v>13463000000</v>
-      </c>
-      <c r="I11" s="16" t="n">
-        <v>14772300000</v>
-      </c>
-      <c r="J11" s="16" t="n">
-        <v>14871000000</v>
-      </c>
-      <c r="K11" s="16" t="n">
-        <v>15752000000</v>
-      </c>
-      <c r="L11" s="16" t="n">
-        <v>15752000000</v>
-      </c>
-      <c r="M11" s="16" t="n">
-        <v>15586000000</v>
-      </c>
-      <c r="N11" s="18" t="n">
         <v>15324000000</v>
       </c>
-      <c r="O11" s="18" t="n">
-        <v>15324000000</v>
-      </c>
-      <c r="P11" s="18" t="n">
-        <v>15324000000</v>
-      </c>
-      <c r="Q11" s="18" t="n">
-        <v>15324000000</v>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>EQUITY</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>EQUITY</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Total Equity</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="16" t="n">
+      <c r="B13" s="17" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="16" t="n">
         <v>508000000</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E13" s="16" t="n">
         <v>729000000</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F13" s="16" t="n">
+        <v>1232400000</v>
+      </c>
+      <c r="G13" s="16" t="n">
         <v>210000000</v>
       </c>
-      <c r="G14" s="16" t="n">
-        <v>1232400000</v>
-      </c>
-      <c r="H14" s="16" t="n">
+      <c r="H13" s="16" t="n">
         <v>4467800000</v>
       </c>
-      <c r="I14" s="16" t="n">
+      <c r="I13" s="16" t="n">
         <v>7230500000</v>
       </c>
-      <c r="J14" s="16" t="n">
+      <c r="J13" s="16" t="n">
+        <v>7824000000</v>
+      </c>
+      <c r="K13" s="16" t="n">
         <v>8665000000</v>
       </c>
-      <c r="K14" s="16" t="n">
+      <c r="L13" s="16" t="n">
         <v>7824000000</v>
       </c>
-      <c r="L14" s="16" t="n">
-        <v>7824000000</v>
-      </c>
-      <c r="M14" s="16" t="n">
+      <c r="M13" s="16" t="n">
         <v>9393000000</v>
       </c>
-      <c r="N14" s="18" t="n">
+      <c r="N13" s="18" t="n">
         <v>10008000000</v>
       </c>
-      <c r="O14" s="18" t="n">
+      <c r="O13" s="18" t="n">
         <v>10623000000</v>
       </c>
-      <c r="P14" s="18" t="n">
+      <c r="P13" s="18" t="n">
         <v>11238000000</v>
       </c>
-      <c r="Q14" s="18" t="n">
+      <c r="Q13" s="18" t="n">
         <v>11853000000</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>BalanceCheck (Assets−Liab−Eq)</t>
         </is>
       </c>
-      <c r="N16" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="23" t="n">
+      <c r="N15" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2171,7 +1932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2296,26 +2057,24 @@
       <c r="B3" s="16" t="n">
         <v>880100000</v>
       </c>
-      <c r="C3" s="16" t="n">
-        <v>2219900000</v>
-      </c>
+      <c r="C3" s="17" t="n"/>
       <c r="D3" s="16" t="n">
+        <v>334000000</v>
+      </c>
+      <c r="E3" s="17" t="n"/>
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="16" t="n">
         <v>351000000</v>
       </c>
-      <c r="E3" s="16" t="n">
-        <v>334000000</v>
-      </c>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="17" t="n"/>
-      <c r="H3" s="17" t="n"/>
-      <c r="I3" s="16" t="n">
+      <c r="H3" s="16" t="n">
         <v>766000000</v>
       </c>
-      <c r="J3" s="17" t="n"/>
+      <c r="I3" s="17" t="n"/>
+      <c r="J3" s="16" t="n">
+        <v>618000000</v>
+      </c>
       <c r="K3" s="17" t="n"/>
-      <c r="L3" s="16" t="n">
-        <v>618000000</v>
-      </c>
+      <c r="L3" s="17" t="n"/>
       <c r="M3" s="17" t="n"/>
       <c r="N3" s="18" t="n">
         <v>0</v>
@@ -2336,23 +2095,25 @@
           <t>Depreciation &amp; Amort</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
+      <c r="B4" s="16" t="n">
+        <v>259600000</v>
+      </c>
       <c r="C4" s="17" t="n"/>
       <c r="D4" s="17" t="n"/>
-      <c r="E4" s="17" t="n"/>
+      <c r="E4" s="16" t="n">
+        <v>84000000</v>
+      </c>
       <c r="F4" s="16" t="n">
-        <v>84000000</v>
-      </c>
-      <c r="G4" s="16" t="n">
         <v>89000000</v>
       </c>
+      <c r="G4" s="17" t="n"/>
       <c r="H4" s="17" t="n"/>
       <c r="I4" s="17" t="n"/>
       <c r="J4" s="17" t="n"/>
-      <c r="K4" s="16" t="n">
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="16" t="n">
         <v>180000000</v>
       </c>
-      <c r="L4" s="17" t="n"/>
       <c r="M4" s="16" t="n">
         <v>171000000</v>
       </c>
@@ -2375,23 +2136,25 @@
           <t>Stock-Based Comp</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
+      <c r="B5" s="16" t="n">
+        <v>940700000</v>
+      </c>
       <c r="C5" s="17" t="n"/>
       <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
+      <c r="E5" s="16" t="n">
+        <v>295000000</v>
+      </c>
       <c r="F5" s="16" t="n">
-        <v>295000000</v>
-      </c>
-      <c r="G5" s="16" t="n">
         <v>370000000</v>
       </c>
+      <c r="G5" s="17" t="n"/>
       <c r="H5" s="17" t="n"/>
       <c r="I5" s="17" t="n"/>
       <c r="J5" s="17" t="n"/>
-      <c r="K5" s="16" t="n">
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="16" t="n">
         <v>671000000</v>
       </c>
-      <c r="L5" s="17" t="n"/>
       <c r="M5" s="16" t="n">
         <v>615000000</v>
       </c>
@@ -2421,24 +2184,26 @@
         <v>-40000000</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>-864400000</v>
+        <v>-165500000</v>
       </c>
       <c r="G6" s="16" t="n">
-        <v>698900000</v>
+        <v>-698900000</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>-271800000</v>
+        <v>427100000</v>
       </c>
       <c r="I6" s="16" t="n">
         <v>-234600000</v>
       </c>
       <c r="J6" s="16" t="n">
-        <v>607000000</v>
+        <v>-1015000000</v>
       </c>
       <c r="K6" s="16" t="n">
+        <v>1622000000</v>
+      </c>
+      <c r="L6" s="16" t="n">
         <v>-1622000000</v>
       </c>
-      <c r="L6" s="17" t="n"/>
       <c r="M6" s="16" t="n">
         <v>849000000</v>
       </c>
@@ -2458,278 +2223,296 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Δ Inventory (−increase)</t>
+          <t>Δ Accounts Payable (+increase)</t>
         </is>
       </c>
       <c r="B7" s="17" t="n"/>
       <c r="C7" s="17" t="n"/>
       <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
+      <c r="E7" s="16" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>-36700000</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>36400000</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>-19100000</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>125900000</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>-2800000</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>-9000000</v>
+      </c>
+      <c r="L7" s="16" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="M7" s="16" t="n">
+        <v>30000000</v>
+      </c>
       <c r="N7" s="18" t="n">
-        <v>-0</v>
+        <v>-262000000</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="P7" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Δ Accounts Payable (+increase)</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="n"/>
+          <t>OPERATING CASH FLOW</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>2695200000</v>
+      </c>
       <c r="C8" s="17" t="n"/>
       <c r="D8" s="17" t="n"/>
       <c r="E8" s="16" t="n">
-        <v>2400000</v>
+        <v>1510000000</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>-300000</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>-36400000</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <v>17300000</v>
-      </c>
-      <c r="I8" s="16" t="n">
-        <v>125900000</v>
-      </c>
-      <c r="J8" s="16" t="n">
-        <v>-11800000</v>
-      </c>
-      <c r="K8" s="16" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="L8" s="17" t="n"/>
+        <v>1771000000</v>
+      </c>
+      <c r="G8" s="17" t="n"/>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="17" t="n"/>
+      <c r="L8" s="16" t="n">
+        <v>2325000000</v>
+      </c>
       <c r="M8" s="16" t="n">
-        <v>30000000</v>
+        <v>2067000000</v>
       </c>
       <c r="N8" s="18" t="n">
-        <v>-262000000</v>
+        <v>2640000000</v>
       </c>
       <c r="O8" s="18" t="n">
-        <v>0</v>
+        <v>786000000</v>
       </c>
       <c r="P8" s="18" t="n">
-        <v>0</v>
+        <v>786000000</v>
       </c>
       <c r="Q8" s="18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>OPERATING CASH FLOW</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="16" t="n">
-        <v>1510000000</v>
-      </c>
-      <c r="G9" s="16" t="n">
-        <v>1771000000</v>
-      </c>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="16" t="n">
-        <v>2325000000</v>
-      </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="16" t="n">
-        <v>2067000000</v>
-      </c>
-      <c r="N9" s="18" t="n">
-        <v>2640000000</v>
-      </c>
-      <c r="O9" s="18" t="n">
         <v>786000000</v>
       </c>
-      <c r="P9" s="18" t="n">
-        <v>786000000</v>
-      </c>
-      <c r="Q9" s="18" t="n">
-        <v>786000000</v>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>INVESTING ACTIVITIES</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>INVESTING ACTIVITIES</t>
-        </is>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Capital Expenditures (−)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>159900000</v>
+      </c>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="16" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>84000000</v>
+      </c>
+      <c r="G11" s="17" t="n"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="17" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="17" t="n"/>
+      <c r="L11" s="16" t="n">
+        <v>254000000</v>
+      </c>
+      <c r="M11" s="16" t="n">
+        <v>92000000</v>
+      </c>
+      <c r="N11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Capital Expenditures (−)</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="n"/>
+          <t>INVESTING CASH FLOW</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>-1442200000</v>
+      </c>
       <c r="C12" s="17" t="n"/>
       <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
+      <c r="E12" s="16" t="n">
+        <v>-544000000</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>-983000000</v>
+      </c>
       <c r="G12" s="17" t="n"/>
       <c r="H12" s="17" t="n"/>
       <c r="I12" s="17" t="n"/>
       <c r="J12" s="17" t="n"/>
       <c r="K12" s="17" t="n"/>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="17" t="n"/>
+      <c r="L12" s="16" t="n">
+        <v>-332000000</v>
+      </c>
+      <c r="M12" s="16" t="n">
+        <v>-925000000</v>
+      </c>
       <c r="N12" s="18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="O12" s="18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="P12" s="18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q12" s="18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>INVESTING CASH FLOW</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="16" t="n">
-        <v>-544000000</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>-983000000</v>
-      </c>
-      <c r="H13" s="17" t="n"/>
-      <c r="I13" s="17" t="n"/>
-      <c r="J13" s="17" t="n"/>
-      <c r="K13" s="16" t="n">
-        <v>-332000000</v>
-      </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="16" t="n">
-        <v>-925000000</v>
-      </c>
-      <c r="N13" s="18" t="n">
         <v>-0</v>
       </c>
-      <c r="O13" s="18" t="n">
-        <v>-0</v>
-      </c>
-      <c r="P13" s="18" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q13" s="18" t="n">
-        <v>-0</v>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>FINANCING ACTIVITIES</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>FINANCING ACTIVITIES</t>
-        </is>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Stock Buybacks (−)</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="17" t="n"/>
+      <c r="K15" s="17" t="n"/>
+      <c r="L15" s="17" t="n"/>
+      <c r="M15" s="17" t="n"/>
+      <c r="N15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Stock Buybacks (−)</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="n"/>
+          <t>FINANCING CASH FLOW</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>-404800000</v>
+      </c>
       <c r="C16" s="17" t="n"/>
       <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
+      <c r="E16" s="16" t="n">
+        <v>-220000000</v>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>8000000</v>
+      </c>
       <c r="G16" s="17" t="n"/>
       <c r="H16" s="17" t="n"/>
       <c r="I16" s="17" t="n"/>
       <c r="J16" s="17" t="n"/>
       <c r="K16" s="17" t="n"/>
-      <c r="L16" s="17" t="n"/>
-      <c r="M16" s="17" t="n"/>
+      <c r="L16" s="16" t="n">
+        <v>-106000000</v>
+      </c>
+      <c r="M16" s="16" t="n">
+        <v>-452000000</v>
+      </c>
       <c r="N16" s="18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="O16" s="18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="P16" s="18" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Q16" s="18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>FINANCING CASH FLOW</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="17" t="n"/>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="16" t="n">
-        <v>-220000000</v>
-      </c>
-      <c r="G17" s="16" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="17" t="n"/>
-      <c r="J17" s="17" t="n"/>
-      <c r="K17" s="16" t="n">
-        <v>-106000000</v>
-      </c>
-      <c r="L17" s="17" t="n"/>
-      <c r="M17" s="16" t="n">
-        <v>-452000000</v>
-      </c>
-      <c r="N17" s="18" t="n">
         <v>-0</v>
       </c>
-      <c r="O17" s="18" t="n">
-        <v>-0</v>
-      </c>
-      <c r="P17" s="18" t="n">
-        <v>-0</v>
-      </c>
-      <c r="Q17" s="18" t="n">
-        <v>-0</v>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Net Change in Cash</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
+      <c r="H18" s="17" t="n"/>
+      <c r="I18" s="17" t="n"/>
+      <c r="J18" s="17" t="n"/>
+      <c r="K18" s="17" t="n"/>
+      <c r="L18" s="17" t="n"/>
+      <c r="M18" s="17" t="n"/>
+      <c r="N18" s="18" t="n">
+        <v>2640000000</v>
+      </c>
+      <c r="O18" s="18" t="n">
+        <v>786000000</v>
+      </c>
+      <c r="P18" s="18" t="n">
+        <v>786000000</v>
+      </c>
+      <c r="Q18" s="18" t="n">
+        <v>786000000</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Net Change in Cash</t>
+          <t>Ending Cash (= BS Cash)</t>
         </is>
       </c>
       <c r="B19" s="17" t="n"/>
@@ -2745,46 +2528,15 @@
       <c r="L19" s="17" t="n"/>
       <c r="M19" s="17" t="n"/>
       <c r="N19" s="18" t="n">
-        <v>2640000000</v>
+        <v>6798000000</v>
       </c>
       <c r="O19" s="18" t="n">
-        <v>786000000</v>
+        <v>7584000000</v>
       </c>
       <c r="P19" s="18" t="n">
-        <v>786000000</v>
+        <v>8370000000</v>
       </c>
       <c r="Q19" s="18" t="n">
-        <v>786000000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Ending Cash (= BS Cash)</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="17" t="n"/>
-      <c r="D20" s="17" t="n"/>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="17" t="n"/>
-      <c r="G20" s="17" t="n"/>
-      <c r="H20" s="17" t="n"/>
-      <c r="I20" s="17" t="n"/>
-      <c r="J20" s="17" t="n"/>
-      <c r="K20" s="17" t="n"/>
-      <c r="L20" s="17" t="n"/>
-      <c r="M20" s="17" t="n"/>
-      <c r="N20" s="18" t="n">
-        <v>6798000000</v>
-      </c>
-      <c r="O20" s="18" t="n">
-        <v>7584000000</v>
-      </c>
-      <c r="P20" s="18" t="n">
-        <v>8370000000</v>
-      </c>
-      <c r="Q20" s="18" t="n">
         <v>9156000000</v>
       </c>
     </row>
@@ -3058,26 +2810,24 @@
       <c r="B4" s="16" t="n">
         <v>6685200000</v>
       </c>
-      <c r="C4" s="16" t="n">
-        <v>5838000000</v>
-      </c>
+      <c r="C4" s="17" t="n"/>
       <c r="D4" s="16" t="n">
+        <v>2474000000</v>
+      </c>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="16" t="n">
         <v>2139000000</v>
       </c>
-      <c r="E4" s="16" t="n">
-        <v>2474000000</v>
-      </c>
-      <c r="F4" s="17" t="n"/>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="17" t="n"/>
-      <c r="I4" s="16" t="n">
+      <c r="H4" s="16" t="n">
         <v>5068000000</v>
       </c>
-      <c r="J4" s="17" t="n"/>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="16" t="n">
+        <v>4396000000</v>
+      </c>
       <c r="K4" s="17" t="n"/>
-      <c r="L4" s="16" t="n">
-        <v>4396000000</v>
-      </c>
+      <c r="L4" s="17" t="n"/>
       <c r="M4" s="17" t="n"/>
       <c r="N4" s="18" t="n">
         <v>0</v>
@@ -3101,26 +2851,24 @@
       <c r="B5" s="16" t="n">
         <v>745700000</v>
       </c>
-      <c r="C5" s="16" t="n">
-        <v>445500000</v>
-      </c>
+      <c r="C5" s="17" t="n"/>
       <c r="D5" s="16" t="n">
+        <v>309000000</v>
+      </c>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="16" t="n">
         <v>286000000</v>
       </c>
-      <c r="E5" s="16" t="n">
-        <v>309000000</v>
-      </c>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="16" t="n">
+      <c r="H5" s="16" t="n">
         <v>706000000</v>
       </c>
-      <c r="J5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="16" t="n">
+        <v>527000000</v>
+      </c>
       <c r="K5" s="17" t="n"/>
-      <c r="L5" s="16" t="n">
-        <v>527000000</v>
-      </c>
+      <c r="L5" s="17" t="n"/>
       <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
         <v>0</v>
@@ -3144,26 +2892,24 @@
       <c r="B6" s="16" t="n">
         <v>880100000</v>
       </c>
-      <c r="C6" s="16" t="n">
-        <v>2219900000</v>
-      </c>
+      <c r="C6" s="17" t="n"/>
       <c r="D6" s="16" t="n">
+        <v>334000000</v>
+      </c>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="16" t="n">
         <v>351000000</v>
       </c>
-      <c r="E6" s="16" t="n">
-        <v>334000000</v>
-      </c>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="16" t="n">
+      <c r="H6" s="16" t="n">
         <v>766000000</v>
       </c>
-      <c r="J6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="16" t="n">
+        <v>618000000</v>
+      </c>
       <c r="K6" s="17" t="n"/>
-      <c r="L6" s="16" t="n">
-        <v>618000000</v>
-      </c>
+      <c r="L6" s="17" t="n"/>
       <c r="M6" s="17" t="n"/>
       <c r="N6" s="18" t="n">
         <v>0</v>
@@ -3184,23 +2930,25 @@
           <t>Operating Cash Flow ($)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
+      <c r="B7" s="16" t="n">
+        <v>2695200000</v>
+      </c>
       <c r="C7" s="17" t="n"/>
       <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
+      <c r="E7" s="16" t="n">
+        <v>1510000000</v>
+      </c>
       <c r="F7" s="16" t="n">
-        <v>1510000000</v>
-      </c>
-      <c r="G7" s="16" t="n">
         <v>1771000000</v>
       </c>
+      <c r="G7" s="17" t="n"/>
       <c r="H7" s="17" t="n"/>
       <c r="I7" s="17" t="n"/>
       <c r="J7" s="17" t="n"/>
-      <c r="K7" s="16" t="n">
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="16" t="n">
         <v>2325000000</v>
       </c>
-      <c r="L7" s="17" t="n"/>
       <c r="M7" s="16" t="n">
         <v>2067000000</v>
       </c>
@@ -3227,7 +2975,7 @@
     <row r="10">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>Max |Modelled OCF − Reported OCF| (last 4Q): $649,000,000  ✗ FAIL (tolerance $5M)</t>
+          <t>Max |Modelled OCF − Reported OCF| (last 4Q): $0  ✓ PASS (tolerance $5M)</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4536,7 @@
         </is>
       </c>
       <c r="C47" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
@@ -4800,12 +4548,12 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4569,7 @@
         </is>
       </c>
       <c r="C48" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
@@ -4833,12 +4581,12 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4602,7 @@
         </is>
       </c>
       <c r="C49" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
@@ -4866,12 +4614,12 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4635,7 @@
         </is>
       </c>
       <c r="C50" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
@@ -4899,12 +4647,12 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -4986,7 +4734,7 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
@@ -4998,12 +4746,12 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -5019,7 +4767,7 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
@@ -5031,12 +4779,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5130,7 @@
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
@@ -5394,12 +5142,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000014</t>
+          <t>0001327567-24-000017</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5163,7 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
@@ -5427,12 +5175,12 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000017</t>
+          <t>0001327567-23-000014</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5427,7 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
@@ -5691,12 +5439,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5460,7 @@
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
@@ -5724,12 +5472,12 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6021,7 @@
         </is>
       </c>
       <c r="C92" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
@@ -6285,12 +6033,12 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000017</t>
+          <t>0001327567-25-000017</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000017/</t>
         </is>
       </c>
     </row>
@@ -6306,7 +6054,7 @@
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
@@ -6318,12 +6066,12 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000017</t>
+          <t>0001327567-24-000017</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000017/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6318,7 @@
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
@@ -6578,16 +6326,16 @@
         </is>
       </c>
       <c r="E101" s="27" t="n">
-        <v>2282800000</v>
+        <v>2283000000</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6351,7 @@
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
@@ -6611,16 +6359,16 @@
         </is>
       </c>
       <c r="E102" s="27" t="n">
-        <v>2283000000</v>
+        <v>2282800000</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6450,7 @@
         </is>
       </c>
       <c r="C105" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
@@ -6710,16 +6458,16 @@
         </is>
       </c>
       <c r="E105" s="27" t="n">
-        <v>1510000000</v>
+        <v>1509600000</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6483,7 @@
         </is>
       </c>
       <c r="C106" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
@@ -6743,16 +6491,16 @@
         </is>
       </c>
       <c r="E106" s="27" t="n">
-        <v>1509600000</v>
+        <v>1510000000</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6582,7 @@
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
@@ -6842,16 +6590,16 @@
         </is>
       </c>
       <c r="E109" s="27" t="n">
-        <v>2139000000</v>
+        <v>2138800000</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6615,7 @@
         </is>
       </c>
       <c r="C110" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
@@ -6875,16 +6623,16 @@
         </is>
       </c>
       <c r="E110" s="27" t="n">
-        <v>2138800000</v>
+        <v>2139000000</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh PANW dashboard artifacts (cash-flow standalone fix)
</commit_message>
<xml_diff>
--- a/dashboard/PANW_3Statement_Model.xlsx
+++ b/dashboard/PANW_3Statement_Model.xlsx
@@ -197,8 +197,8 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -607,7 +607,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-05-24</t>
+          <t>Generated: 2026-05-28</t>
         </is>
       </c>
     </row>
@@ -811,13 +811,13 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>-0.2</v>
+        <v>0.04</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>-0.3</v>
+        <v>0.06</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>-0.08000000000000002</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="3">
@@ -827,13 +827,13 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.68</v>
+        <v>0.7377161055505005</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>0.6936000000000001</v>
+        <v>0.7524704276615105</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>0.6664</v>
+        <v>0.7229617834394905</v>
       </c>
     </row>
     <row r="4">
@@ -843,13 +843,13 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>-0.2</v>
+        <v>-0.1062849621586048</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>-0.16</v>
+        <v>-0.08502796972688387</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>-0.26</v>
+        <v>-0.1381704508061863</v>
       </c>
     </row>
     <row r="5">
@@ -875,13 +875,13 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>60</v>
+        <v>60.70291173794358</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>57</v>
+        <v>57.6677661510464</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>66</v>
+        <v>66.77320291173794</v>
       </c>
     </row>
     <row r="7">
@@ -891,13 +891,13 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>45</v>
+        <v>18.10928013876843</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>45</v>
+        <v>18.10928013876843</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>45</v>
+        <v>18.10928013876843</v>
       </c>
     </row>
     <row r="8">
@@ -955,13 +955,13 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>-0.2</v>
+        <v>0.04</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>0.68</v>
+        <v>0.7377161055505005</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -1072,7 +1072,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>-0.2</v>
+        <v>-0.1062849621586048</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>60</v>
+        <v>60.70291173794358</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>45</v>
+        <v>18.10928013876843</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -1331,41 +1331,37 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B2" s="16" t="n">
-        <v>6685200000</v>
-      </c>
-      <c r="C2" s="16" t="n">
-        <v>5838000000</v>
-      </c>
-      <c r="D2" s="16" t="n">
+      <c r="B2" s="16" t="n"/>
+      <c r="C2" s="16" t="n"/>
+      <c r="D2" s="16" t="n"/>
+      <c r="E2" s="17" t="n">
         <v>2139000000</v>
       </c>
-      <c r="E2" s="16" t="n">
+      <c r="F2" s="16" t="n"/>
+      <c r="G2" s="17" t="n">
         <v>2474000000</v>
       </c>
-      <c r="F2" s="17" t="n"/>
-      <c r="G2" s="17" t="n"/>
-      <c r="H2" s="17" t="n"/>
-      <c r="I2" s="16" t="n">
+      <c r="H2" s="16" t="n"/>
+      <c r="I2" s="16" t="n"/>
+      <c r="J2" s="16" t="n"/>
+      <c r="K2" s="16" t="n"/>
+      <c r="L2" s="17" t="n">
         <v>5068000000</v>
       </c>
-      <c r="J2" s="17" t="n"/>
-      <c r="K2" s="17" t="n"/>
-      <c r="L2" s="16" t="n">
+      <c r="M2" s="17" t="n">
         <v>4396000000</v>
       </c>
-      <c r="M2" s="17" t="n"/>
       <c r="N2" s="18" t="n">
-        <v>0</v>
+        <v>4571840000</v>
       </c>
       <c r="O2" s="18" t="n">
-        <v>0</v>
+        <v>4754713600</v>
       </c>
       <c r="P2" s="18" t="n">
-        <v>0</v>
+        <v>4944902144</v>
       </c>
       <c r="Q2" s="18" t="n">
-        <v>0</v>
+        <v>5142698229.76</v>
       </c>
     </row>
     <row r="3">
@@ -1374,41 +1370,37 @@
           <t>Cost of Revenue</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
-        <v>1772600000</v>
-      </c>
-      <c r="C3" s="16" t="n">
-        <v>1485500000</v>
-      </c>
-      <c r="D3" s="16" t="n">
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="17" t="n">
         <v>554000000</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="17" t="n">
         <v>638000000</v>
       </c>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="17" t="n"/>
-      <c r="H3" s="17" t="n"/>
-      <c r="I3" s="16" t="n">
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
+      <c r="J3" s="16" t="n"/>
+      <c r="K3" s="16" t="n"/>
+      <c r="L3" s="17" t="n">
         <v>1323000000</v>
       </c>
-      <c r="J3" s="17" t="n"/>
-      <c r="K3" s="17" t="n"/>
-      <c r="L3" s="16" t="n">
+      <c r="M3" s="17" t="n">
         <v>1153000000</v>
       </c>
-      <c r="M3" s="17" t="n"/>
       <c r="N3" s="18" t="n">
-        <v>0</v>
+        <v>1199120000</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>0</v>
+        <v>1247084800</v>
       </c>
       <c r="P3" s="18" t="n">
-        <v>0</v>
+        <v>1296968192</v>
       </c>
       <c r="Q3" s="18" t="n">
-        <v>0</v>
+        <v>1348846919.68</v>
       </c>
     </row>
     <row r="4">
@@ -1417,41 +1409,37 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
-        <v>4912600000</v>
-      </c>
-      <c r="C4" s="16" t="n">
-        <v>4352500000</v>
-      </c>
-      <c r="D4" s="16" t="n">
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n">
         <v>1585000000</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="17" t="n">
         <v>1836000000</v>
       </c>
-      <c r="F4" s="17" t="n"/>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="17" t="n"/>
-      <c r="I4" s="16" t="n">
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="17" t="n">
         <v>3745000000</v>
       </c>
-      <c r="J4" s="17" t="n"/>
-      <c r="K4" s="17" t="n"/>
-      <c r="L4" s="16" t="n">
+      <c r="M4" s="17" t="n">
         <v>3243000000</v>
       </c>
-      <c r="M4" s="17" t="n"/>
       <c r="N4" s="18" t="n">
-        <v>0</v>
+        <v>3372720000</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>0</v>
+        <v>3507628800</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>0</v>
+        <v>3647933952</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>0</v>
+        <v>3793851310.08</v>
       </c>
     </row>
     <row r="5">
@@ -1460,41 +1448,37 @@
           <t>Operating Expenses</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>4166900000</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>3907000000</v>
-      </c>
-      <c r="D5" s="16" t="n">
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="17" t="n">
         <v>1299000000</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="17" t="n">
         <v>1527000000</v>
       </c>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="16" t="n">
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="17" t="n">
         <v>3039000000</v>
       </c>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="16" t="n">
+      <c r="M5" s="17" t="n">
         <v>2716000000</v>
       </c>
-      <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
-        <v>0</v>
+        <v>2427330042.777229</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>0</v>
+        <v>2169341361.034207</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>0</v>
+        <v>1938772996.56759</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>0</v>
+        <v>1732710581.993279</v>
       </c>
     </row>
     <row r="6">
@@ -1503,41 +1487,37 @@
           <t>Operating Income</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
-        <v>745700000</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>445500000</v>
-      </c>
-      <c r="D6" s="16" t="n">
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="17" t="n">
         <v>286000000</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="17" t="n">
         <v>309000000</v>
       </c>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="16" t="n">
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="17" t="n">
         <v>706000000</v>
       </c>
-      <c r="J6" s="17" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="16" t="n">
+      <c r="M6" s="17" t="n">
         <v>527000000</v>
       </c>
-      <c r="M6" s="17" t="n"/>
       <c r="N6" s="18" t="n">
-        <v>0</v>
+        <v>945389957.2227707</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>0</v>
+        <v>1338287438.965793</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>0</v>
+        <v>1709160955.43241</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>0</v>
+        <v>2061140728.086722</v>
       </c>
     </row>
     <row r="7">
@@ -1546,41 +1526,37 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
-        <v>880100000</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>2219900000</v>
-      </c>
-      <c r="D7" s="16" t="n">
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="17" t="n">
         <v>351000000</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="17" t="n">
         <v>334000000</v>
       </c>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="16" t="n">
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="17" t="n">
         <v>766000000</v>
       </c>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="16" t="n">
+      <c r="M7" s="17" t="n">
         <v>618000000</v>
       </c>
-      <c r="M7" s="17" t="n"/>
       <c r="N7" s="18" t="n">
-        <v>0</v>
+        <v>803581463.6393551</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>0</v>
+        <v>1137544323.120924</v>
       </c>
       <c r="P7" s="18" t="n">
-        <v>0</v>
+        <v>1452786812.117548</v>
       </c>
       <c r="Q7" s="18" t="n">
-        <v>0</v>
+        <v>1751969618.873713</v>
       </c>
     </row>
     <row r="9">
@@ -1589,35 +1565,29 @@
           <t>Gross Margin %</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n">
-        <v>0.7348471249925208</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>0.7455464200068517</v>
-      </c>
-      <c r="D9" s="19" t="n">
+      <c r="E9" s="19" t="n">
         <v>0.7410004675081814</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="G9" s="19" t="n">
         <v>0.7421180274858529</v>
       </c>
-      <c r="I9" s="19" t="n">
+      <c r="L9" s="19" t="n">
         <v>0.738950276243094</v>
       </c>
-      <c r="L9" s="19" t="n">
+      <c r="M9" s="19" t="n">
         <v>0.7377161055505005</v>
       </c>
       <c r="N9" s="20" t="n">
-        <v>0</v>
+        <v>0.7377161055505005</v>
       </c>
       <c r="O9" s="20" t="n">
-        <v>0</v>
+        <v>0.7377161055505005</v>
       </c>
       <c r="P9" s="20" t="n">
-        <v>0</v>
+        <v>0.7377161055505005</v>
       </c>
       <c r="Q9" s="20" t="n">
-        <v>0</v>
+        <v>0.7377161055505005</v>
       </c>
     </row>
   </sheetData>
@@ -1745,49 +1715,49 @@
           <t>Cash &amp; Equivalents</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="16" t="n">
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="17" t="n">
         <v>2067200000</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="E3" s="17" t="n">
         <v>1346300000</v>
       </c>
-      <c r="F3" s="16" t="n">
+      <c r="F3" s="17" t="n">
         <v>2118500000</v>
       </c>
-      <c r="G3" s="16" t="n">
+      <c r="G3" s="17" t="n">
         <v>1992900000</v>
       </c>
-      <c r="H3" s="16" t="n">
+      <c r="H3" s="17" t="n">
         <v>1373700000</v>
       </c>
-      <c r="I3" s="16" t="n">
+      <c r="I3" s="17" t="n">
         <v>2383400000</v>
       </c>
-      <c r="J3" s="16" t="n">
+      <c r="J3" s="17" t="n">
+        <v>2269000000</v>
+      </c>
+      <c r="K3" s="17" t="n">
         <v>3066000000</v>
       </c>
-      <c r="K3" s="16" t="n">
+      <c r="L3" s="17" t="n">
+        <v>4158000000</v>
+      </c>
+      <c r="M3" s="17" t="n">
         <v>2269000000</v>
       </c>
-      <c r="L3" s="16" t="n">
-        <v>2269000000</v>
-      </c>
-      <c r="M3" s="16" t="n">
-        <v>4158000000</v>
-      </c>
       <c r="N3" s="18" t="n">
-        <v>6798000000</v>
+        <v>2958689623.639355</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>7584000000</v>
+        <v>3977786433.160279</v>
       </c>
       <c r="P3" s="18" t="n">
-        <v>8370000000</v>
+        <v>5307387831.133827</v>
       </c>
       <c r="Q3" s="18" t="n">
-        <v>9156000000</v>
+        <v>6931244619.297781</v>
       </c>
     </row>
     <row r="4">
@@ -1796,49 +1766,49 @@
           <t>Accounts Receivable</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="17" t="n"/>
-      <c r="D4" s="16" t="n">
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="17" t="n">
         <v>1238100000</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="E4" s="17" t="n">
         <v>1278100000</v>
       </c>
-      <c r="F4" s="16" t="n">
+      <c r="F4" s="17" t="n">
         <v>2142500000</v>
       </c>
-      <c r="G4" s="16" t="n">
+      <c r="G4" s="17" t="n">
         <v>1443600000</v>
       </c>
-      <c r="H4" s="16" t="n">
+      <c r="H4" s="17" t="n">
         <v>1715400000</v>
       </c>
-      <c r="I4" s="16" t="n">
+      <c r="I4" s="17" t="n">
         <v>1950000000</v>
       </c>
-      <c r="J4" s="16" t="n">
+      <c r="J4" s="17" t="n">
+        <v>2965000000</v>
+      </c>
+      <c r="K4" s="17" t="n">
         <v>1343000000</v>
       </c>
-      <c r="K4" s="16" t="n">
+      <c r="L4" s="17" t="n">
+        <v>2116000000</v>
+      </c>
+      <c r="M4" s="17" t="n">
         <v>2965000000</v>
       </c>
-      <c r="L4" s="16" t="n">
-        <v>2965000000</v>
-      </c>
-      <c r="M4" s="16" t="n">
-        <v>2116000000</v>
-      </c>
       <c r="N4" s="18" t="n">
-        <v>0</v>
+        <v>3083600000</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>0</v>
+        <v>3206944000</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>0</v>
+        <v>3335221760</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>0</v>
+        <v>3468630630.4</v>
       </c>
     </row>
     <row r="5">
@@ -1847,18 +1817,18 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="n"/>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="16" t="n"/>
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="16" t="n"/>
+      <c r="M5" s="16" t="n"/>
       <c r="N5" s="18" t="n">
         <v>0</v>
       </c>
@@ -1878,49 +1848,49 @@
           <t>TOTAL ASSETS</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="16" t="n">
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="17" t="n">
         <v>12543800000</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="17" t="n">
         <v>13163400000</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <v>12253600000</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="17" t="n">
         <v>14170500000</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>17930800000</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="17" t="n">
         <v>22002800000</v>
       </c>
-      <c r="J6" s="16" t="n">
+      <c r="J6" s="17" t="n">
+        <v>23576000000</v>
+      </c>
+      <c r="K6" s="17" t="n">
         <v>23536000000</v>
       </c>
-      <c r="K6" s="16" t="n">
+      <c r="L6" s="17" t="n">
+        <v>24979000000</v>
+      </c>
+      <c r="M6" s="17" t="n">
         <v>23576000000</v>
       </c>
-      <c r="L6" s="16" t="n">
-        <v>23576000000</v>
-      </c>
-      <c r="M6" s="16" t="n">
-        <v>24979000000</v>
-      </c>
       <c r="N6" s="18" t="n">
-        <v>25332000000</v>
+        <v>24388861463.63935</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>25947000000</v>
+        <v>25536056986.76028</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>26562000000</v>
+        <v>26998881046.87783</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>27177000000</v>
+        <v>28761289403.67154</v>
       </c>
     </row>
     <row r="8">
@@ -1936,49 +1906,49 @@
           <t>Accounts Payable</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="16" t="n">
+      <c r="B9" s="16" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="17" t="n">
         <v>125900000</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="17" t="n">
         <v>128300000</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="17" t="n">
         <v>128000000</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="17" t="n">
         <v>91600000</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="17" t="n">
         <v>108900000</v>
       </c>
-      <c r="I9" s="16" t="n">
+      <c r="I9" s="17" t="n">
         <v>234800000</v>
       </c>
-      <c r="J9" s="16" t="n">
+      <c r="J9" s="17" t="n">
+        <v>232000000</v>
+      </c>
+      <c r="K9" s="17" t="n">
         <v>223000000</v>
       </c>
-      <c r="K9" s="16" t="n">
+      <c r="L9" s="17" t="n">
+        <v>262000000</v>
+      </c>
+      <c r="M9" s="17" t="n">
         <v>232000000</v>
       </c>
-      <c r="L9" s="16" t="n">
-        <v>232000000</v>
-      </c>
-      <c r="M9" s="16" t="n">
-        <v>262000000</v>
-      </c>
       <c r="N9" s="18" t="n">
-        <v>0</v>
+        <v>241280000</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>0</v>
+        <v>250931200</v>
       </c>
       <c r="P9" s="18" t="n">
-        <v>0</v>
+        <v>260968448</v>
       </c>
       <c r="Q9" s="18" t="n">
-        <v>0</v>
+        <v>271407185.92</v>
       </c>
     </row>
     <row r="10">
@@ -1987,49 +1957,49 @@
           <t>Deferred Revenue</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="16" t="n">
+      <c r="B10" s="16" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="17" t="n">
         <v>3741300000</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="17" t="n">
         <v>3942500000</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="17" t="n">
         <v>3641200000</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="17" t="n">
         <v>4146700000</v>
       </c>
-      <c r="H10" s="16" t="n">
+      <c r="H10" s="17" t="n">
         <v>5014900000</v>
       </c>
-      <c r="I10" s="16" t="n">
+      <c r="I10" s="17" t="n">
         <v>5756800000</v>
       </c>
-      <c r="J10" s="16" t="n">
+      <c r="J10" s="17" t="n">
+        <v>6302000000</v>
+      </c>
+      <c r="K10" s="17" t="n">
         <v>6132000000</v>
       </c>
-      <c r="K10" s="16" t="n">
+      <c r="L10" s="17" t="n">
+        <v>6248000000</v>
+      </c>
+      <c r="M10" s="17" t="n">
         <v>6302000000</v>
       </c>
-      <c r="L10" s="16" t="n">
+      <c r="N10" s="18" t="n">
         <v>6302000000</v>
       </c>
-      <c r="M10" s="16" t="n">
-        <v>6248000000</v>
-      </c>
-      <c r="N10" s="18" t="n">
-        <v>6248000000</v>
-      </c>
       <c r="O10" s="18" t="n">
-        <v>6248000000</v>
+        <v>6302000000</v>
       </c>
       <c r="P10" s="18" t="n">
-        <v>6248000000</v>
+        <v>6302000000</v>
       </c>
       <c r="Q10" s="18" t="n">
-        <v>6248000000</v>
+        <v>6302000000</v>
       </c>
     </row>
     <row r="11">
@@ -2038,49 +2008,49 @@
           <t>TOTAL LIABILITIES</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n"/>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="16" t="n">
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="17" t="n">
         <v>12035800000</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="17" t="n">
         <v>12434400000</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="17" t="n">
         <v>12043600000</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="17" t="n">
         <v>12938100000</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="17" t="n">
         <v>13463000000</v>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="I11" s="17" t="n">
         <v>14772300000</v>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="J11" s="17" t="n">
+        <v>15752000000</v>
+      </c>
+      <c r="K11" s="17" t="n">
         <v>14871000000</v>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="L11" s="17" t="n">
+        <v>15586000000</v>
+      </c>
+      <c r="M11" s="17" t="n">
         <v>15752000000</v>
       </c>
-      <c r="L11" s="16" t="n">
-        <v>15752000000</v>
-      </c>
-      <c r="M11" s="16" t="n">
-        <v>15586000000</v>
-      </c>
       <c r="N11" s="18" t="n">
-        <v>15324000000</v>
+        <v>15761280000</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>15324000000</v>
+        <v>15770931200</v>
       </c>
       <c r="P11" s="18" t="n">
-        <v>15324000000</v>
+        <v>15780968448</v>
       </c>
       <c r="Q11" s="18" t="n">
-        <v>15324000000</v>
+        <v>15791407185.92</v>
       </c>
     </row>
     <row r="13">
@@ -2096,49 +2066,49 @@
           <t>Total Equity</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="16" t="n">
+      <c r="B14" s="16" t="n"/>
+      <c r="C14" s="16" t="n"/>
+      <c r="D14" s="17" t="n">
         <v>508000000</v>
       </c>
-      <c r="E14" s="16" t="n">
+      <c r="E14" s="17" t="n">
         <v>729000000</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="17" t="n">
         <v>210000000</v>
       </c>
-      <c r="G14" s="16" t="n">
+      <c r="G14" s="17" t="n">
         <v>1232400000</v>
       </c>
-      <c r="H14" s="16" t="n">
+      <c r="H14" s="17" t="n">
         <v>4467800000</v>
       </c>
-      <c r="I14" s="16" t="n">
+      <c r="I14" s="17" t="n">
         <v>7230500000</v>
       </c>
-      <c r="J14" s="16" t="n">
+      <c r="J14" s="17" t="n">
+        <v>7824000000</v>
+      </c>
+      <c r="K14" s="17" t="n">
         <v>8665000000</v>
       </c>
-      <c r="K14" s="16" t="n">
+      <c r="L14" s="17" t="n">
+        <v>9393000000</v>
+      </c>
+      <c r="M14" s="17" t="n">
         <v>7824000000</v>
       </c>
-      <c r="L14" s="16" t="n">
-        <v>7824000000</v>
-      </c>
-      <c r="M14" s="16" t="n">
-        <v>9393000000</v>
-      </c>
       <c r="N14" s="18" t="n">
-        <v>10008000000</v>
+        <v>8627581463.639355</v>
       </c>
       <c r="O14" s="18" t="n">
-        <v>10623000000</v>
+        <v>9765125786.760279</v>
       </c>
       <c r="P14" s="18" t="n">
-        <v>11238000000</v>
+        <v>11217912598.87783</v>
       </c>
       <c r="Q14" s="18" t="n">
-        <v>11853000000</v>
+        <v>12969882217.75154</v>
       </c>
     </row>
     <row r="16">
@@ -2151,13 +2121,13 @@
         <v>0</v>
       </c>
       <c r="O16" s="23" t="n">
-        <v>0</v>
+        <v>-1.9073486328125e-06</v>
       </c>
       <c r="P16" s="23" t="n">
         <v>0</v>
       </c>
       <c r="Q16" s="23" t="n">
-        <v>0</v>
+        <v>-1.9073486328125e-06</v>
       </c>
     </row>
   </sheetData>
@@ -2293,41 +2263,37 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B3" s="16" t="n">
-        <v>880100000</v>
-      </c>
-      <c r="C3" s="16" t="n">
-        <v>2219900000</v>
-      </c>
-      <c r="D3" s="16" t="n">
+      <c r="B3" s="16" t="n"/>
+      <c r="C3" s="16" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="17" t="n">
         <v>351000000</v>
       </c>
-      <c r="E3" s="16" t="n">
+      <c r="F3" s="16" t="n"/>
+      <c r="G3" s="17" t="n">
         <v>334000000</v>
       </c>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="17" t="n"/>
-      <c r="H3" s="17" t="n"/>
-      <c r="I3" s="16" t="n">
+      <c r="H3" s="16" t="n"/>
+      <c r="I3" s="16" t="n"/>
+      <c r="J3" s="16" t="n"/>
+      <c r="K3" s="16" t="n"/>
+      <c r="L3" s="17" t="n">
         <v>766000000</v>
       </c>
-      <c r="J3" s="17" t="n"/>
-      <c r="K3" s="17" t="n"/>
-      <c r="L3" s="16" t="n">
+      <c r="M3" s="17" t="n">
         <v>618000000</v>
       </c>
-      <c r="M3" s="17" t="n"/>
       <c r="N3" s="18" t="n">
-        <v>0</v>
+        <v>803581463.6393551</v>
       </c>
       <c r="O3" s="18" t="n">
-        <v>0</v>
+        <v>1137544323.120924</v>
       </c>
       <c r="P3" s="18" t="n">
-        <v>0</v>
+        <v>1452786812.117548</v>
       </c>
       <c r="Q3" s="18" t="n">
-        <v>0</v>
+        <v>1751969618.873713</v>
       </c>
     </row>
     <row r="4">
@@ -2336,37 +2302,41 @@
           <t>Depreciation &amp; Amort</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="17" t="n"/>
-      <c r="D4" s="17" t="n"/>
-      <c r="E4" s="17" t="n"/>
-      <c r="F4" s="16" t="n">
+      <c r="B4" s="17" t="n">
+        <v>259600000</v>
+      </c>
+      <c r="C4" s="17" t="n">
+        <v>207200000</v>
+      </c>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n">
+        <v>89000000</v>
+      </c>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="17" t="n">
         <v>84000000</v>
       </c>
-      <c r="G4" s="16" t="n">
-        <v>89000000</v>
-      </c>
-      <c r="H4" s="17" t="n"/>
-      <c r="I4" s="17" t="n"/>
-      <c r="J4" s="17" t="n"/>
-      <c r="K4" s="16" t="n">
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="17" t="n">
         <v>180000000</v>
       </c>
-      <c r="L4" s="17" t="n"/>
-      <c r="M4" s="16" t="n">
+      <c r="L4" s="17" t="n">
         <v>171000000</v>
       </c>
+      <c r="M4" s="16" t="n"/>
       <c r="N4" s="18" t="n">
-        <v>171000000</v>
+        <v>0</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>171000000</v>
+        <v>0</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>171000000</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>171000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -2375,37 +2345,41 @@
           <t>Stock-Based Comp</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n"/>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="16" t="n">
+      <c r="B5" s="17" t="n">
+        <v>940700000</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>806500000</v>
+      </c>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="17" t="n">
+        <v>370000000</v>
+      </c>
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="17" t="n">
         <v>295000000</v>
       </c>
-      <c r="G5" s="16" t="n">
-        <v>370000000</v>
-      </c>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="16" t="n">
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="17" t="n">
         <v>671000000</v>
       </c>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="16" t="n">
+      <c r="L5" s="17" t="n">
         <v>615000000</v>
       </c>
+      <c r="M5" s="16" t="n"/>
       <c r="N5" s="18" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>615000000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2414,45 +2388,47 @@
           <t>Δ Accounts Receivable (−increase)</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="16" t="n">
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="17" t="n">
         <v>-40000000</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <v>-864400000</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="17" t="n">
         <v>698900000</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>-271800000</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="17" t="n">
         <v>-234600000</v>
       </c>
-      <c r="J6" s="16" t="n">
-        <v>607000000</v>
-      </c>
-      <c r="K6" s="16" t="n">
-        <v>-1622000000</v>
-      </c>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="16" t="n">
-        <v>849000000</v>
+      <c r="J6" s="17" t="n">
+        <v>-1015000000</v>
+      </c>
+      <c r="K6" s="17" t="n">
+        <v>1622000000</v>
+      </c>
+      <c r="L6" s="17" t="n">
+        <v>-773000000</v>
+      </c>
+      <c r="M6" s="17" t="n">
+        <v>-849000000</v>
       </c>
       <c r="N6" s="18" t="n">
-        <v>2116000000</v>
+        <v>-118600000</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>-0</v>
+        <v>-123344000</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>-0</v>
+        <v>-128277760</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>-0</v>
+        <v>-133408870.4000001</v>
       </c>
     </row>
     <row r="7">
@@ -2461,18 +2437,18 @@
           <t>Δ Inventory (−increase)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
+      <c r="B7" s="16" t="n"/>
+      <c r="C7" s="16" t="n"/>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="16" t="n"/>
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
+      <c r="M7" s="16" t="n"/>
       <c r="N7" s="18" t="n">
         <v>-0</v>
       </c>
@@ -2492,45 +2468,47 @@
           <t>Δ Accounts Payable (+increase)</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n"/>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="16" t="n">
+      <c r="B8" s="16" t="n"/>
+      <c r="C8" s="16" t="n"/>
+      <c r="D8" s="16" t="n"/>
+      <c r="E8" s="17" t="n">
         <v>2400000</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="17" t="n">
         <v>-300000</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="17" t="n">
         <v>-36400000</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="17" t="n">
         <v>17300000</v>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I8" s="17" t="n">
         <v>125900000</v>
       </c>
-      <c r="J8" s="16" t="n">
-        <v>-11800000</v>
-      </c>
-      <c r="K8" s="16" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="16" t="n">
-        <v>30000000</v>
+      <c r="J8" s="17" t="n">
+        <v>-2800000</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>-9000000</v>
+      </c>
+      <c r="L8" s="17" t="n">
+        <v>39000000</v>
+      </c>
+      <c r="M8" s="17" t="n">
+        <v>-30000000</v>
       </c>
       <c r="N8" s="18" t="n">
-        <v>-262000000</v>
+        <v>9279999.99999997</v>
       </c>
       <c r="O8" s="18" t="n">
-        <v>0</v>
+        <v>9651200</v>
       </c>
       <c r="P8" s="18" t="n">
-        <v>0</v>
+        <v>10037248</v>
       </c>
       <c r="Q8" s="18" t="n">
-        <v>0</v>
+        <v>10438737.91999999</v>
       </c>
     </row>
     <row r="9">
@@ -2539,37 +2517,41 @@
           <t>OPERATING CASH FLOW</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n"/>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="16" t="n">
+      <c r="B9" s="17" t="n">
+        <v>2695200000</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>2744900000</v>
+      </c>
+      <c r="D9" s="16" t="n"/>
+      <c r="E9" s="17" t="n">
+        <v>1771000000</v>
+      </c>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="17" t="n">
         <v>1510000000</v>
       </c>
-      <c r="G9" s="16" t="n">
-        <v>1771000000</v>
-      </c>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="16" t="n">
+      <c r="H9" s="16" t="n"/>
+      <c r="I9" s="16" t="n"/>
+      <c r="J9" s="16" t="n"/>
+      <c r="K9" s="17" t="n">
         <v>2325000000</v>
       </c>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="16" t="n">
+      <c r="L9" s="17" t="n">
         <v>2067000000</v>
       </c>
+      <c r="M9" s="16" t="n"/>
       <c r="N9" s="18" t="n">
-        <v>2640000000</v>
+        <v>694261463.6393551</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>786000000</v>
+        <v>1023851523.120924</v>
       </c>
       <c r="P9" s="18" t="n">
-        <v>786000000</v>
+        <v>1334546300.117548</v>
       </c>
       <c r="Q9" s="18" t="n">
-        <v>786000000</v>
+        <v>1628999486.393713</v>
       </c>
     </row>
     <row r="11">
@@ -2585,29 +2567,29 @@
           <t>Capital Expenditures (−)</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n"/>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="17" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="17" t="n"/>
-      <c r="K12" s="17" t="n"/>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="17" t="n"/>
+      <c r="B12" s="16" t="n"/>
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="16" t="n"/>
+      <c r="H12" s="16" t="n"/>
+      <c r="I12" s="16" t="n"/>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="16" t="n"/>
+      <c r="L12" s="16" t="n"/>
+      <c r="M12" s="16" t="n"/>
       <c r="N12" s="18" t="n">
-        <v>0</v>
+        <v>4571840</v>
       </c>
       <c r="O12" s="18" t="n">
-        <v>0</v>
+        <v>4754713.600000001</v>
       </c>
       <c r="P12" s="18" t="n">
-        <v>0</v>
+        <v>4944902.144</v>
       </c>
       <c r="Q12" s="18" t="n">
-        <v>0</v>
+        <v>5142698.22976</v>
       </c>
     </row>
     <row r="13">
@@ -2616,37 +2598,41 @@
           <t>INVESTING CASH FLOW</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n"/>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="16" t="n">
+      <c r="B13" s="17" t="n">
+        <v>-1442200000</v>
+      </c>
+      <c r="C13" s="17" t="n">
+        <v>-1341400000</v>
+      </c>
+      <c r="D13" s="16" t="n"/>
+      <c r="E13" s="17" t="n">
+        <v>-983000000</v>
+      </c>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="17" t="n">
         <v>-544000000</v>
       </c>
-      <c r="G13" s="16" t="n">
-        <v>-983000000</v>
-      </c>
-      <c r="H13" s="17" t="n"/>
-      <c r="I13" s="17" t="n"/>
-      <c r="J13" s="17" t="n"/>
-      <c r="K13" s="16" t="n">
+      <c r="H13" s="16" t="n"/>
+      <c r="I13" s="16" t="n"/>
+      <c r="J13" s="16" t="n"/>
+      <c r="K13" s="17" t="n">
         <v>-332000000</v>
       </c>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="16" t="n">
+      <c r="L13" s="17" t="n">
         <v>-925000000</v>
       </c>
+      <c r="M13" s="16" t="n"/>
       <c r="N13" s="18" t="n">
-        <v>-0</v>
+        <v>-4571840</v>
       </c>
       <c r="O13" s="18" t="n">
-        <v>-0</v>
+        <v>-4754713.600000001</v>
       </c>
       <c r="P13" s="18" t="n">
-        <v>-0</v>
+        <v>-4944902.144</v>
       </c>
       <c r="Q13" s="18" t="n">
-        <v>-0</v>
+        <v>-5142698.22976</v>
       </c>
     </row>
     <row r="15">
@@ -2662,18 +2648,20 @@
           <t>Stock Buybacks (−)</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="17" t="n"/>
-      <c r="I16" s="17" t="n"/>
-      <c r="J16" s="17" t="n"/>
-      <c r="K16" s="17" t="n"/>
-      <c r="L16" s="17" t="n"/>
-      <c r="M16" s="17" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="17" t="n">
+        <v>566700000</v>
+      </c>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="16" t="n"/>
+      <c r="H16" s="16" t="n"/>
+      <c r="I16" s="16" t="n"/>
+      <c r="J16" s="16" t="n"/>
+      <c r="K16" s="16" t="n"/>
+      <c r="L16" s="16" t="n"/>
+      <c r="M16" s="16" t="n"/>
       <c r="N16" s="18" t="n">
         <v>0</v>
       </c>
@@ -2693,26 +2681,30 @@
           <t>FINANCING CASH FLOW</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="17" t="n"/>
-      <c r="D17" s="17" t="n"/>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="16" t="n">
+      <c r="B17" s="17" t="n">
+        <v>-404800000</v>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>-1163800000</v>
+      </c>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="17" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="17" t="n">
         <v>-220000000</v>
       </c>
-      <c r="G17" s="16" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="H17" s="17" t="n"/>
-      <c r="I17" s="17" t="n"/>
-      <c r="J17" s="17" t="n"/>
-      <c r="K17" s="16" t="n">
+      <c r="H17" s="16" t="n"/>
+      <c r="I17" s="16" t="n"/>
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="17" t="n">
         <v>-106000000</v>
       </c>
-      <c r="L17" s="17" t="n"/>
-      <c r="M17" s="16" t="n">
+      <c r="L17" s="17" t="n">
         <v>-452000000</v>
       </c>
+      <c r="M17" s="16" t="n"/>
       <c r="N17" s="18" t="n">
         <v>-0</v>
       </c>
@@ -2732,29 +2724,29 @@
           <t>Net Change in Cash</t>
         </is>
       </c>
-      <c r="B19" s="17" t="n"/>
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="17" t="n"/>
-      <c r="H19" s="17" t="n"/>
-      <c r="I19" s="17" t="n"/>
-      <c r="J19" s="17" t="n"/>
-      <c r="K19" s="17" t="n"/>
-      <c r="L19" s="17" t="n"/>
-      <c r="M19" s="17" t="n"/>
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="16" t="n"/>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="16" t="n"/>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="16" t="n"/>
+      <c r="I19" s="16" t="n"/>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="16" t="n"/>
+      <c r="L19" s="16" t="n"/>
+      <c r="M19" s="16" t="n"/>
       <c r="N19" s="18" t="n">
-        <v>2640000000</v>
+        <v>689689623.6393551</v>
       </c>
       <c r="O19" s="18" t="n">
-        <v>786000000</v>
+        <v>1019096809.520924</v>
       </c>
       <c r="P19" s="18" t="n">
-        <v>786000000</v>
+        <v>1329601397.973548</v>
       </c>
       <c r="Q19" s="18" t="n">
-        <v>786000000</v>
+        <v>1623856788.163954</v>
       </c>
     </row>
     <row r="20">
@@ -2763,29 +2755,29 @@
           <t>Ending Cash (= BS Cash)</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n"/>
-      <c r="C20" s="17" t="n"/>
-      <c r="D20" s="17" t="n"/>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="17" t="n"/>
-      <c r="G20" s="17" t="n"/>
-      <c r="H20" s="17" t="n"/>
-      <c r="I20" s="17" t="n"/>
-      <c r="J20" s="17" t="n"/>
-      <c r="K20" s="17" t="n"/>
-      <c r="L20" s="17" t="n"/>
-      <c r="M20" s="17" t="n"/>
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="16" t="n"/>
+      <c r="E20" s="16" t="n"/>
+      <c r="F20" s="16" t="n"/>
+      <c r="G20" s="16" t="n"/>
+      <c r="H20" s="16" t="n"/>
+      <c r="I20" s="16" t="n"/>
+      <c r="J20" s="16" t="n"/>
+      <c r="K20" s="16" t="n"/>
+      <c r="L20" s="16" t="n"/>
+      <c r="M20" s="16" t="n"/>
       <c r="N20" s="18" t="n">
-        <v>6798000000</v>
+        <v>2958689623.639355</v>
       </c>
       <c r="O20" s="18" t="n">
-        <v>7584000000</v>
+        <v>3977786433.160279</v>
       </c>
       <c r="P20" s="18" t="n">
-        <v>8370000000</v>
+        <v>5307387831.133827</v>
       </c>
       <c r="Q20" s="18" t="n">
-        <v>9156000000</v>
+        <v>6931244619.297781</v>
       </c>
     </row>
   </sheetData>
@@ -3055,41 +3047,37 @@
           <t>Revenue ($)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
-        <v>6685200000</v>
-      </c>
-      <c r="C4" s="16" t="n">
-        <v>5838000000</v>
-      </c>
-      <c r="D4" s="16" t="n">
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n">
         <v>2139000000</v>
       </c>
-      <c r="E4" s="16" t="n">
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="17" t="n">
         <v>2474000000</v>
       </c>
-      <c r="F4" s="17" t="n"/>
-      <c r="G4" s="17" t="n"/>
-      <c r="H4" s="17" t="n"/>
-      <c r="I4" s="16" t="n">
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="17" t="n">
         <v>5068000000</v>
       </c>
-      <c r="J4" s="17" t="n"/>
-      <c r="K4" s="17" t="n"/>
-      <c r="L4" s="16" t="n">
+      <c r="M4" s="17" t="n">
         <v>4396000000</v>
       </c>
-      <c r="M4" s="17" t="n"/>
       <c r="N4" s="18" t="n">
-        <v>0</v>
+        <v>4571840000</v>
       </c>
       <c r="O4" s="18" t="n">
-        <v>0</v>
+        <v>4754713600</v>
       </c>
       <c r="P4" s="18" t="n">
-        <v>0</v>
+        <v>4944902144</v>
       </c>
       <c r="Q4" s="18" t="n">
-        <v>0</v>
+        <v>5142698229.76</v>
       </c>
     </row>
     <row r="5">
@@ -3098,41 +3086,37 @@
           <t>Operating Income ($)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>745700000</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>445500000</v>
-      </c>
-      <c r="D5" s="16" t="n">
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="17" t="n">
         <v>286000000</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="F5" s="16" t="n"/>
+      <c r="G5" s="17" t="n">
         <v>309000000</v>
       </c>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="16" t="n">
+      <c r="H5" s="16" t="n"/>
+      <c r="I5" s="16" t="n"/>
+      <c r="J5" s="16" t="n"/>
+      <c r="K5" s="16" t="n"/>
+      <c r="L5" s="17" t="n">
         <v>706000000</v>
       </c>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="16" t="n">
+      <c r="M5" s="17" t="n">
         <v>527000000</v>
       </c>
-      <c r="M5" s="17" t="n"/>
       <c r="N5" s="18" t="n">
-        <v>0</v>
+        <v>945389957.2227707</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>0</v>
+        <v>1338287438.965793</v>
       </c>
       <c r="P5" s="18" t="n">
-        <v>0</v>
+        <v>1709160955.43241</v>
       </c>
       <c r="Q5" s="18" t="n">
-        <v>0</v>
+        <v>2061140728.086722</v>
       </c>
     </row>
     <row r="6">
@@ -3141,41 +3125,37 @@
           <t>Net Income ($)</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
-        <v>880100000</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>2219900000</v>
-      </c>
-      <c r="D6" s="16" t="n">
+      <c r="B6" s="16" t="n"/>
+      <c r="C6" s="16" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="17" t="n">
         <v>351000000</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="F6" s="16" t="n"/>
+      <c r="G6" s="17" t="n">
         <v>334000000</v>
       </c>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="16" t="n">
+      <c r="H6" s="16" t="n"/>
+      <c r="I6" s="16" t="n"/>
+      <c r="J6" s="16" t="n"/>
+      <c r="K6" s="16" t="n"/>
+      <c r="L6" s="17" t="n">
         <v>766000000</v>
       </c>
-      <c r="J6" s="17" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="16" t="n">
+      <c r="M6" s="17" t="n">
         <v>618000000</v>
       </c>
-      <c r="M6" s="17" t="n"/>
       <c r="N6" s="18" t="n">
-        <v>0</v>
+        <v>803581463.6393551</v>
       </c>
       <c r="O6" s="18" t="n">
-        <v>0</v>
+        <v>1137544323.120924</v>
       </c>
       <c r="P6" s="18" t="n">
-        <v>0</v>
+        <v>1452786812.117548</v>
       </c>
       <c r="Q6" s="18" t="n">
-        <v>0</v>
+        <v>1751969618.873713</v>
       </c>
     </row>
     <row r="7">
@@ -3184,37 +3164,41 @@
           <t>Operating Cash Flow ($)</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n"/>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="16" t="n">
+      <c r="B7" s="17" t="n">
+        <v>2695200000</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>2744900000</v>
+      </c>
+      <c r="D7" s="16" t="n"/>
+      <c r="E7" s="17" t="n">
+        <v>1771000000</v>
+      </c>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="17" t="n">
         <v>1510000000</v>
       </c>
-      <c r="G7" s="16" t="n">
-        <v>1771000000</v>
-      </c>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="16" t="n">
+      <c r="H7" s="16" t="n"/>
+      <c r="I7" s="16" t="n"/>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="17" t="n">
         <v>2325000000</v>
       </c>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="16" t="n">
+      <c r="L7" s="17" t="n">
         <v>2067000000</v>
       </c>
+      <c r="M7" s="16" t="n"/>
       <c r="N7" s="18" t="n">
-        <v>2640000000</v>
+        <v>694261463.6393551</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>786000000</v>
+        <v>1023851523.120924</v>
       </c>
       <c r="P7" s="18" t="n">
-        <v>786000000</v>
+        <v>1334546300.117548</v>
       </c>
       <c r="Q7" s="18" t="n">
-        <v>786000000</v>
+        <v>1628999486.393713</v>
       </c>
     </row>
     <row r="9">
@@ -3227,7 +3211,7 @@
     <row r="10">
       <c r="A10" s="26" t="inlineStr">
         <is>
-          <t>Max |Modelled OCF − Reported OCF| (last 4Q): $649,000,000  ✗ FAIL (tolerance $5M)</t>
+          <t>Max |Modelled OCF − Reported OCF| (last 4Q): $2,299,000,000  ✗ FAIL (tolerance $5M)</t>
         </is>
       </c>
     </row>
@@ -4986,7 +4970,7 @@
         </is>
       </c>
       <c r="C53" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
@@ -4998,12 +4982,12 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>0001327567-22-000038</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5003,7 @@
         </is>
       </c>
       <c r="C54" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
@@ -5031,12 +5015,12 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-22-000038</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756722000038/</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5366,7 @@
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
@@ -5394,12 +5378,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000014</t>
+          <t>0001327567-24-000017</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5399,7 @@
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
@@ -5427,12 +5411,12 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000017</t>
+          <t>0001327567-23-000014</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000017/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000014/</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5663,7 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
@@ -5691,12 +5675,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5696,7 @@
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
@@ -5724,12 +5708,12 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -5745,7 +5729,7 @@
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
@@ -5757,12 +5741,12 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>0001327567-23-000032</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5762,7 @@
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
@@ -5790,12 +5774,12 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-23-000032</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756723000032/</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6752,7 @@
         </is>
       </c>
       <c r="C107" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
@@ -6776,16 +6760,16 @@
         </is>
       </c>
       <c r="E107" s="27" t="n">
-        <v>286500000</v>
+        <v>286000000</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>
@@ -6801,7 +6785,7 @@
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
@@ -6809,16 +6793,16 @@
         </is>
       </c>
       <c r="E108" s="27" t="n">
-        <v>286000000</v>
+        <v>286500000</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6834,7 +6818,7 @@
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
@@ -6842,16 +6826,16 @@
         </is>
       </c>
       <c r="E109" s="27" t="n">
-        <v>2139000000</v>
+        <v>2138800000</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>0001327567-25-000035</t>
+          <t>0001327567-24-000040</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
         </is>
       </c>
     </row>
@@ -6867,7 +6851,7 @@
         </is>
       </c>
       <c r="C110" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
@@ -6875,16 +6859,16 @@
         </is>
       </c>
       <c r="E110" s="27" t="n">
-        <v>2138800000</v>
+        <v>2139000000</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>0001327567-24-000040</t>
+          <t>0001327567-25-000035</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756724000040/</t>
+          <t>https://www.sec.gov/Archives/edgar/data/1327567/000132756725000035/</t>
         </is>
       </c>
     </row>

</xml_diff>